<commit_message>
[ADD] Implementation of CSV format feature to upload the sales order for market places sales.
</commit_message>
<xml_diff>
--- a/home_kouzina_sales/static/src/files/sale_order_template.xlsx
+++ b/home_kouzina_sales/static/src/files/sale_order_template.xlsx
@@ -8,7 +8,8 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sale Order Template" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Import Report" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -20,15 +21,86 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
-  <si>
-    <t xml:space="preserve">Customer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Product Code</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+  <si>
+    <t xml:space="preserve">Marketplace Order ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Order Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customer Email</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Billing Street</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Billing City</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Billing State</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Billing Zip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Currency</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Product </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="JetBrains Mono"/>
+        <family val="3"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">SKU</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Product Name</t>
   </si>
   <si>
     <t xml:space="preserve">Quantity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unit Price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tax Percent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shipping Amount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Order Line Note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Order Tag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Rows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Created Orders</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Failed Rows</t>
   </si>
 </sst>
 </file>
@@ -38,7 +110,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -62,35 +134,39 @@
       <family val="0"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Cambria"/>
-      <family val="0"/>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
       <charset val="1"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4F81BD"/>
+        <bgColor rgb="FF4BACC6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4BACC6"/>
+        <bgColor rgb="FF4F81BD"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -134,7 +210,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -143,19 +219,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -168,6 +240,66 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF4BACC6"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF4F81BD"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -351,13 +483,21 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:Q1048576"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="1" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="15.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="26.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="5" style="1" width="15.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="26.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="12" style="1" width="15.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="19.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="15.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="10.16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -367,64 +507,104 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="4" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
+      <c r="A2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="5"/>
+      <c r="A3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>

</xml_diff>